<commit_message>
Add view counts and subscriber counts to analysis sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHN5v8daos2wujZ76BPAyH
</commit_message>
<xml_diff>
--- a/youtube-world-history-research/output/video_analysis_sheet.xlsx
+++ b/youtube-world-history-research/output/video_analysis_sheet.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -63,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -72,6 +74,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -442,17 +450,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,30 +479,45 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>登録者数</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>動画タイトル</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>動画URL</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>再生数</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>再生数÷登録者数</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>誰に向けた動画か</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>見たら何が得られると約束しているか</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>どんな感情を動かしているか（驚き・不安・好奇心など）</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>サムネの構図・文字数・色・人物の表情</t>
         </is>
@@ -508,20 +534,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>なぜ最強だったはずのモンゴル帝国は ヨーロッパを侵略できなかったのか？【歴史解説】</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=y0cwR7ttIaY</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="n">
+        <v>549553</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="6" t="inlineStr"/>
+      <c r="J2" s="6" t="inlineStr"/>
+      <c r="K2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -534,20 +569,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>【立場逆転】侵略しに来たのに狩られる側に…モンゴル目線で見る元寇の恐怖【歴史解説】</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=t_Kje4VAKiE</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="4" t="inlineStr"/>
-      <c r="G3" s="4" t="inlineStr"/>
-      <c r="H3" s="4" t="inlineStr"/>
+      <c r="F3" s="4" t="n">
+        <v>1299382</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -560,20 +604,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>【恐怖】日本のバケモン海賊「倭寇」、さすがに厄介すぎる【歴史解説】</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=62_F5SjtZCM</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr"/>
-      <c r="F4" s="4" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr"/>
-      <c r="H4" s="4" t="inlineStr"/>
+      <c r="F4" s="4" t="n">
+        <v>741800</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="6" t="inlineStr"/>
+      <c r="K4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -586,20 +639,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>街角の子供から戦場の兵士まで...世界を支配したコカ・コーラの歴史【歴史解説】</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=e-i5fvSbPM0</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="n">
+        <v>278564</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -612,20 +674,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>【総集編】犯罪者が建国し、凡ミスで滅亡...歴史上存在したヤバすぎる国たち【歴史解説】</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=_CE6EZ7nBWY</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="4" t="inlineStr"/>
-      <c r="G6" s="4" t="inlineStr"/>
-      <c r="H6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="n">
+        <v>409355</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="inlineStr"/>
+      <c r="K6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -638,20 +709,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>【致〇率99%】敵陣に最初に突入する兵士のモチベーションは何だったのか？【歴史解説】</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=lOGdA7_YDe0</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
-      <c r="G7" s="4" t="inlineStr"/>
-      <c r="H7" s="4" t="inlineStr"/>
+      <c r="F7" s="4" t="n">
+        <v>3214321</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="inlineStr"/>
+      <c r="K7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -664,20 +744,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>ビックリするほどしょーもない理由で滅亡した国３選【歴史解説】</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=EXsFtJWLtLw</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="4" t="inlineStr"/>
-      <c r="H8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="n">
+        <v>414461</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="inlineStr"/>
+      <c r="K8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -690,20 +779,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>なぜ攻撃力最強のはずの機関銃は、軍人たちから嫌われまくっていたのか？【歴史解説】</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=oqU0VDyQiUE</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="n">
+        <v>317807</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="6" t="inlineStr"/>
+      <c r="K9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -716,20 +814,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>「歩兵」が中世ヨーロッパの戦場を”地獄”に変えたと言われる理由【歴史解説】</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=mMzDpd9NA38</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="n">
+        <v>1516503</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr"/>
+      <c r="K10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -742,20 +849,29 @@
           <t>https://www.youtube.com/@sekaishi_ura</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="n">
+        <v>263000</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>防御力最強のはずの「城塞都市」が日本で採用されなかった意外な理由【歴史解説】</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=ebAl58P2JRc</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr"/>
-      <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="n">
+        <v>3164917</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="6" t="inlineStr"/>
+      <c r="K11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -768,20 +884,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>なぜインドは「人口世界一」になったのか？14億人を生んだ最強の地形と残酷な歴史</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=sky5rp3O0fg</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="n">
+        <v>14759</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="6" t="inlineStr"/>
+      <c r="K12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -794,20 +919,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>【驚愕の地理】日本より細長い国が存在した！？チリ・ノルウェー・ベトナムが抱える過酷な宿命と驚きの共通点</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=_rEy7JfXiKE</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr"/>
-      <c r="H13" s="4" t="inlineStr"/>
+      <c r="F13" s="4" t="n">
+        <v>10723</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr"/>
+      <c r="K13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -820,20 +954,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>【大人の歴史物語】なぜ北米の巨大な島「グリーンランド」は、遠く離れたデンマーク領なのか？ 〜嘘と勘違いから始まった数奇な運命〜</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=b8Hy-06K0mY</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr"/>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="4" t="inlineStr"/>
-      <c r="H14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="n">
+        <v>43346</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="6" t="inlineStr"/>
+      <c r="K14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -846,20 +989,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>【地政学と歴史】中国はなぜ日本海に出られないのか？ロシアに奪われた「15kmの壁」の真実</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=0fQNhKQyVcg</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="n">
+        <v>9957</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="6" t="inlineStr"/>
+      <c r="K15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -872,20 +1024,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>なぜ中央アジアは「5つのスタン」に分かれたのか？【シルクロードの真実】</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=L1HApBYXYaw</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="n">
+        <v>145756</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr"/>
+      <c r="K16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -898,20 +1059,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>ロシア最大の痛恨…なぜ「世界最大の宝の山」を手放したのか？坪単価0.2円で売られたアラスカの悲劇と歴史の皮肉</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=YgU5vvbNHFc</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="n">
+        <v>117755</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="6" t="inlineStr"/>
+      <c r="K17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -924,20 +1094,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>一見すると双子なのに…オランダとベルギーはなぜ「別の国」になったのか？【引き裂かれた歴史】</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=WTxwe4d4qXM</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr"/>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="n">
+        <v>231422</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="6" t="inlineStr"/>
+      <c r="K18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -950,20 +1129,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>国旗も言葉もほぼ同じなのに…北欧が「一つの国」になれなかった理由</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=rJqy3SXia3Y</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="n">
+        <v>376231</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="6" t="inlineStr"/>
+      <c r="K19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -976,20 +1164,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>一つ屋根の下に二つの家族？イベリア半島が「２つに分かれた」歴史の裏側</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=dkrkDvQjz-4</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr"/>
-      <c r="F20" s="4" t="inlineStr"/>
-      <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="n">
+        <v>221200</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr"/>
+      <c r="K20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1002,20 +1199,29 @@
           <t>https://www.youtube.com/@%E3%81%8A%E3%82%82%E3%81%97%E3%82%8D%E4%B8%96%E7%95%8C%E5%8F%B2%E3%83%A9%E3%83%9C</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="4" t="n">
+        <v>7160</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>同じ言語なのに、なぜ別の国？ドイツとオーストリアの複雑すぎる愛憎史</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=MIE3-uo--r4</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr"/>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="4" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr"/>
+      <c r="F21" s="4" t="n">
+        <v>174273</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="H21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr"/>
+      <c r="K21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1028,20 +1234,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>ヘルマン・ゲーリング｜残酷すぎる最期。53歳で死去したヒトラーの後継者【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=BtAGQokhyUE</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr"/>
-      <c r="G22" s="4" t="inlineStr"/>
-      <c r="H22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="n">
+        <v>81175</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H22" s="6" t="inlineStr"/>
+      <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="6" t="inlineStr"/>
+      <c r="K22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1054,20 +1269,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>イルマ・グレーゼ｜22歳で処刑された悪魔。ナチスが最も恐れた女の残酷すぎる最期【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=XBXVSbh4w1k</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr"/>
-      <c r="F23" s="4" t="inlineStr"/>
-      <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="n">
+        <v>576986</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>29.4</v>
+      </c>
+      <c r="H23" s="6" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr"/>
+      <c r="K23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1080,20 +1304,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>ラインハルト・ハイドリヒ｜数百万人を虐殺した悪魔。ナチスが最も恐れた男の残酷すぎる最期【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=K4AcedCAqj4</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr"/>
-      <c r="F24" s="4" t="inlineStr"/>
-      <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="n">
+        <v>147795</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H24" s="6" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="6" t="inlineStr"/>
+      <c r="K24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1106,20 +1339,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>毛沢東の最期！4500万人を殺した男の残酷すぎる44日間【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=UdZXaobRj_U</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="n">
+        <v>184827</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H25" s="6" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="6" t="inlineStr"/>
+      <c r="K25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1132,20 +1374,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>ラヴレンチー・ベリヤ｜数百万人を虐殺した悪魔。スターリンが絶賛したソ連の秘密警察長官【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=6KhwEtMg3-M</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr"/>
-      <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="n">
+        <v>108893</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="H26" s="6" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="6" t="inlineStr"/>
+      <c r="K26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1158,20 +1409,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>エルヴィン・ロンメル｜ヒトラーに殺された男。伝説の無敵将校「砂漠の狐」の残酷すぎる最期【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=b0K8lXRPE_g</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
-      <c r="G27" s="4" t="inlineStr"/>
-      <c r="H27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="n">
+        <v>184439</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H27" s="6" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="6" t="inlineStr"/>
+      <c r="K27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1184,20 +1444,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>アドルフ・アイヒマン｜500万人を殺した男。ナチスが最も恐れた男の残酷すぎる最期【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=bHrzNTlZntI</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr"/>
-      <c r="F28" s="4" t="inlineStr"/>
-      <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="n">
+        <v>245871</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H28" s="6" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr"/>
+      <c r="J28" s="6" t="inlineStr"/>
+      <c r="K28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1210,20 +1479,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>スターリンの最期！1000万人を殺した男の残酷すぎる7日間【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=Rqgbenusa_8</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr"/>
-      <c r="F29" s="4" t="inlineStr"/>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
+      <c r="F29" s="4" t="n">
+        <v>510806</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="H29" s="6" t="inlineStr"/>
+      <c r="I29" s="6" t="inlineStr"/>
+      <c r="J29" s="6" t="inlineStr"/>
+      <c r="K29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1236,20 +1514,29 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>ムッソリーニの最期！逆さ吊りで公開処刑されるまでの残酷すぎる10日間【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=ANxbHSdWPUg</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="4" t="inlineStr"/>
-      <c r="G30" s="4" t="inlineStr"/>
-      <c r="H30" s="4" t="inlineStr"/>
+      <c r="F30" s="4" t="n">
+        <v>210398</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H30" s="6" t="inlineStr"/>
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="6" t="inlineStr"/>
+      <c r="K30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1262,83 +1549,92 @@
           <t>https://www.youtube.com/@hello-senjo</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C31" s="4" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>ヒトラーの最期！最恐独裁者の悲惨すぎる最後の48時間【第二次世界大戦】</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=PINVVV6JeGg</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="n">
+        <v>243970</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="H31" s="6" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="6" t="inlineStr"/>
+      <c r="K31" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Label view and subscriber columns with their dates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHN5v8daos2wujZ76BPAyH
</commit_message>
<xml_diff>
--- a/youtube-world-history-research/output/video_analysis_sheet.xlsx
+++ b/youtube-world-history-research/output/video_analysis_sheet.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>登録者数</t>
+          <t>登録者数（10/8〜9時点）</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>再生数</t>
+          <t>再生数（10/15時点）</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">

</xml_diff>